<commit_message>
Deploy sales_tracker_2b.xlsx to 2B Sales OS
</commit_message>
<xml_diff>
--- a/sales_tracker_2b.xlsx
+++ b/sales_tracker_2b.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abdallah.ahmed\Desktop\plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A3C1195-0079-47BB-9ED6-D6696DD3220E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{467A9196-39AF-4593-AADD-D0399AD13317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-117" yWindow="-117" windowWidth="25142" windowHeight="13544" activeTab="3" xr2:uid="{34265437-78C7-42DF-B49C-D8392DBFC400}"/>
+    <workbookView xWindow="-117" yWindow="-117" windowWidth="25142" windowHeight="13544" activeTab="3" xr2:uid="{5BED53FD-1141-4193-A96F-A745F2DCB422}"/>
   </bookViews>
   <sheets>
-    <sheet name="توزيع التارجت (3.7M)" sheetId="1" r:id="rId1"/>
-    <sheet name="خطة الـ 90 يوماً للمندوبين" sheetId="2" r:id="rId2"/>
-    <sheet name="فصول عام 2027 (36.8M)" sheetId="3" r:id="rId3"/>
+    <sheet name="توزيع الكوارتر (3.7M)" sheetId="1" r:id="rId1"/>
+    <sheet name="شهور الكوارتر الـ 3 (90 يوماً)" sheetId="2" r:id="rId2"/>
+    <sheet name="كوارترات عام 2027 (14.8M)" sheetId="3" r:id="rId3"/>
     <sheet name="حوافز المندوبين والميدان" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -37,21 +37,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="79">
   <si>
     <t>القناة / المسؤول التجاري</t>
   </si>
   <si>
-    <t>المناطق ونوعية العملاء</t>
-  </si>
-  <si>
-    <t>التارجت الأساسي</t>
-  </si>
-  <si>
-    <t>حصة التوسع (+1.5M)</t>
-  </si>
-  <si>
-    <t>التارجت الشهري الكلي</t>
+    <t>المناطق والعملاء المستهدفين</t>
+  </si>
+  <si>
+    <t>أساس الكوارتر</t>
+  </si>
+  <si>
+    <t>توسع الكوارتر (+1.5M)</t>
+  </si>
+  <si>
+    <t>تارجت الكوارتر الكلي</t>
   </si>
   <si>
     <t>مستهدف الكاش (50%)</t>
@@ -63,7 +63,7 @@
     <t>سقف الآجل (50%)</t>
   </si>
   <si>
-    <t>طبيعة المعايرة</t>
+    <t>المعادل الشهري</t>
   </si>
   <si>
     <t>كبار الموزعين والجملة (بإشراف ASM)</t>
@@ -72,37 +72,28 @@
     <t>كبار تجار الجملة ومعارض الكمبيوتر</t>
   </si>
   <si>
-    <t>67.5% - الكتلة الحجمية الأكبر</t>
-  </si>
-  <si>
     <t>مندوب 1 (Zone 1 - شمال الجيزة)</t>
   </si>
   <si>
     <t>المهندسين، الدقي، إمبابة، الوراق</t>
   </si>
   <si>
-    <t>يبدأ بـ 350K في الشهر الأول</t>
-  </si>
-  <si>
     <t>مندوب 2 (Zone 2 - جنوب الجيزة)</t>
   </si>
   <si>
     <t>فيصل، الهرم، 6 أكتوبر، الشيخ زايد</t>
   </si>
   <si>
-    <t>إجمالي قطاع الجيزة الكبرى</t>
-  </si>
-  <si>
-    <t>كامل قطاعات التجزئة والجملة</t>
-  </si>
-  <si>
-    <t>36.8 مليون ج.م سنوياً لعام 2027</t>
-  </si>
-  <si>
-    <t>الشهر التشغيلي</t>
-  </si>
-  <si>
-    <t>كبار الموزعين والجملة</t>
+    <t>إجمالي تارجت الكوارتر (3 شهور)</t>
+  </si>
+  <si>
+    <t>كامل قطاع الجيزة ومحاور التوسع</t>
+  </si>
+  <si>
+    <t>الشهر في الكوارتر</t>
+  </si>
+  <si>
+    <t>كبار الموزعين (ASM)</t>
   </si>
   <si>
     <t>تارجت مندوب 1</t>
@@ -111,48 +102,45 @@
     <t>تارجت مندوب 2</t>
   </si>
   <si>
-    <t>إجمالي تارجت الجيزة</t>
-  </si>
-  <si>
-    <t>معدل النمو</t>
+    <t>إجمالي تارجت الشهر</t>
+  </si>
+  <si>
+    <t>الوزن النسبي %</t>
   </si>
   <si>
     <t>المعالم التشغيلية والمهام الميدانية</t>
   </si>
   <si>
-    <t>الشهر الأول (تأسيس وتعارف)</t>
-  </si>
-  <si>
-    <t>نزول ميداني مزدوج، 8-10 زيارات يومياً، وفتح 8 عملاء جدد كاش لكل مندوب</t>
-  </si>
-  <si>
-    <t>الشهر الثاني (توسع وتكرار)</t>
-  </si>
-  <si>
-    <t>تكرار سحب المحلات القائمة، تركيب وحدات الكاونتر، وتدوير فواتير الآجل (10K)</t>
-  </si>
-  <si>
-    <t>الشهر الثالث (استقرار كامل)</t>
-  </si>
-  <si>
-    <t>استقلالية المندوبين بنسبة 100%، واكتمال المستهدف التوسعي كاملاً (+1.5M)</t>
-  </si>
-  <si>
-    <t>الربع السنوي (2027)</t>
+    <t>الشهر الأول (تأسيس وتجديد)</t>
+  </si>
+  <si>
+    <t>مسح 100% من خطوط السير وتأهيل المناديب وفتح 8 عملاء جدد كاش</t>
+  </si>
+  <si>
+    <t>الشهر الثاني (تسارع وتوسع)</t>
+  </si>
+  <si>
+    <t>إطلاق باقات اللابتوب والشواحن وتركيب 20 ستاند وتدوير الآجل (14 يوماً)</t>
+  </si>
+  <si>
+    <t>الشهر الثالث (ذروة وإغلاق)</t>
+  </si>
+  <si>
+    <t>اكتمال تارجت الكوارتر بالكامل (3.7M)، وتصفية التحصيلات وحساب الحوافز</t>
+  </si>
+  <si>
+    <t>الربع السنوي (الكوارتر)</t>
   </si>
   <si>
     <t>شهور الربع</t>
   </si>
   <si>
-    <t>المستهدف المالي</t>
+    <t>مستهدف الكوارتر</t>
   </si>
   <si>
     <t>المتوسط الشهري</t>
   </si>
   <si>
-    <t>الوزن النسبي %</t>
-  </si>
-  <si>
     <t>المحرك التجاري والموسم</t>
   </si>
   <si>
@@ -162,7 +150,7 @@
     <t>يناير - مارس</t>
   </si>
   <si>
-    <t>تجديد مخزون التجار بعد الجرد السنوي وإجازة منتصف العام</t>
+    <t>تجديد مخزون التجار بعد الجرد السنوي وإجازة منتصف العام وبداية الترم الثاني</t>
   </si>
   <si>
     <t>Q2 (الربع الثاني)</t>
@@ -171,7 +159,7 @@
     <t>أبريل - يونيو</t>
   </si>
   <si>
-    <t>مواسم الأعياد، حركة المصايف، وباور بانك السعات الكبيرة</t>
+    <t>مواسم الأعياد، انطلاق حركة المصايف، وباور بانك وشواحن السفر والسيارات</t>
   </si>
   <si>
     <t>Q3 (الربع الثالث - الذهبي)</t>
@@ -180,7 +168,7 @@
     <t>يوليو - سبتمبر</t>
   </si>
   <si>
-    <t>موسم الجامعات والمدارس: شنط لابتوب وماوس ومحولات Hubs</t>
+    <t>موسم الجامعات والمدارس (Back to School): حزم اللابتوب والشنط والمحولات</t>
   </si>
   <si>
     <t>Q4 (الربع الرابع - الذروة)</t>
@@ -189,16 +177,16 @@
     <t>أكتوبر - ديسمبر</t>
   </si>
   <si>
-    <t>عروض البلاك فرايداي وإغلاق التعاقدات السنوية وتصفية التحصيلات</t>
-  </si>
-  <si>
-    <t>إجمالي عام 2027 الكامل</t>
+    <t>عروض الجمعة البيضاء وإغلاق المستهدفات السنوية وتصفية التحصيلات</t>
+  </si>
+  <si>
+    <t>إجمالي عام 2027 (4 كوارترات)</t>
   </si>
   <si>
     <t>12 شهراً</t>
   </si>
   <si>
-    <t>مستهدف سنوي مدروس وواقعي لقطاع الجيزة (+28% نمو)</t>
+    <t>مستهدف سنوي متوازن ومدروس لقطاع الجيزة (14,800,000 ج.م)</t>
   </si>
   <si>
     <t>بند الحافز والمكافأة</t>
@@ -246,28 +234,31 @@
     <t>حماية السيولة ومنع تعثر الأموال في السوق</t>
   </si>
   <si>
-    <t>بونص تحقيق التارجت الكامل (100%)</t>
-  </si>
-  <si>
-    <t>4,500 ج.م</t>
-  </si>
-  <si>
-    <t>تحقيق 600,000 ج.م شهرياً</t>
-  </si>
-  <si>
-    <t>مكافأة الاستقرار البيعي الكامل للمندوب</t>
-  </si>
-  <si>
-    <t>بونص نجم الشهر (Super Star 110%+)</t>
-  </si>
-  <si>
-    <t>6,500 ج.م + درع تميز</t>
-  </si>
-  <si>
-    <t>تحقيق &gt; 660,000 ج.م</t>
-  </si>
-  <si>
-    <t>إشعال روح التنافس الإيجابي بين المندوبين</t>
+    <t>بونص تحقيق تارجت الكوارتر (100%)</t>
+  </si>
+  <si>
+    <t>13,500 ج.م</t>
+  </si>
+  <si>
+    <t>تحقيق 600,000 ج.م في الكوارتر</t>
+  </si>
+  <si>
+    <t>ربع سنوي</t>
+  </si>
+  <si>
+    <t>مكافأة الاستقرار البيعي الكامل للمندوب (بواقع 4,500 ج.م شهرياً)</t>
+  </si>
+  <si>
+    <t>بونص نجم الكوارتر (Super Star 110%+)</t>
+  </si>
+  <si>
+    <t>19,500 ج.م + درع تميز</t>
+  </si>
+  <si>
+    <t>تحقيق &gt; 660,000 ج.م في الكوارتر</t>
+  </si>
+  <si>
+    <t>إشعال روح التنافس الإيجابي بين المندوبين طوال الـ 3 شهور</t>
   </si>
   <si>
     <t>شنطة الاستبدال الفوري للتالف (RMA)</t>
@@ -677,19 +668,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D343AA0-55EF-4FC3-9873-A783B9332CD6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B624F405-C3B3-4C25-B291-4B21606C2BC0}">
   <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="14.95" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="16.25" x14ac:dyDescent="0.3">
@@ -749,16 +740,17 @@
         <f>E2*0.5</f>
         <v>1250000</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>11</v>
+      <c r="I2" s="3">
+        <f>E2/3</f>
+        <v>833333.33333333337</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="C3" s="3">
         <v>200000</v>
@@ -781,16 +773,17 @@
         <f>E3*0.5</f>
         <v>300000</v>
       </c>
-      <c r="I3" s="2" t="s">
-        <v>14</v>
+      <c r="I3" s="3">
+        <f>E3/3</f>
+        <v>200000</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3">
         <v>200000</v>
@@ -813,16 +806,17 @@
         <f>E4*0.5</f>
         <v>300000</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>14</v>
+      <c r="I4" s="3">
+        <f>E4/3</f>
+        <v>200000</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C5" s="3">
         <f>SUM(C2:C4)</f>
@@ -847,8 +841,9 @@
         <f>SUM(H2:H4)</f>
         <v>1850000</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>19</v>
+      <c r="I5" s="3">
+        <f>E5/3</f>
+        <v>1233333.3333333333</v>
       </c>
     </row>
   </sheetData>
@@ -857,111 +852,111 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB25697E-69EA-49EB-A8E7-6E9C06999F22}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F14A4C6B-5CE6-4A0C-8131-420AC4E566A9}">
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.95" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="62.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="59.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B2" s="3">
-        <v>2000000</v>
+        <v>700000</v>
       </c>
       <c r="C2" s="3">
-        <v>350000</v>
+        <v>150000</v>
       </c>
       <c r="D2" s="3">
-        <v>350000</v>
+        <v>150000</v>
       </c>
       <c r="E2" s="3">
         <f>SUM(B2:D2)</f>
-        <v>2700000</v>
+        <v>1000000</v>
       </c>
       <c r="F2" s="4">
-        <v>0.22700000000000001</v>
+        <v>0.27</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B3" s="3">
-        <v>2300000</v>
+        <v>850000</v>
       </c>
       <c r="C3" s="3">
-        <v>450000</v>
+        <v>225000</v>
       </c>
       <c r="D3" s="3">
-        <v>450000</v>
+        <v>225000</v>
       </c>
       <c r="E3" s="3">
         <f>SUM(B3:D3)</f>
-        <v>3200000</v>
+        <v>1300000</v>
       </c>
       <c r="F3" s="4">
-        <v>0.185</v>
+        <v>0.35099999999999998</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B4" s="3">
-        <v>2500000</v>
+        <v>950000</v>
       </c>
       <c r="C4" s="3">
-        <v>600000</v>
+        <v>225000</v>
       </c>
       <c r="D4" s="3">
-        <v>600000</v>
+        <v>225000</v>
       </c>
       <c r="E4" s="3">
         <f>SUM(B4:D4)</f>
-        <v>3700000</v>
+        <v>1400000</v>
       </c>
       <c r="F4" s="4">
-        <v>0.156</v>
+        <v>0.379</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -970,143 +965,143 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49BA7E44-C106-4D1A-9B17-39D1A159D734}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{864ABE96-EDFB-4AC4-ABEC-5DCDE12150D2}">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.95" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="54.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="63.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="E1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C2" s="3">
-        <v>7500000</v>
+        <v>3400000</v>
       </c>
       <c r="D2" s="3">
         <f>C2/3</f>
-        <v>2500000</v>
+        <v>1133333.3333333333</v>
       </c>
       <c r="E2" s="4">
-        <v>0.20399999999999999</v>
+        <v>0.23</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C3" s="3">
-        <v>9000000</v>
+        <v>3700000</v>
       </c>
       <c r="D3" s="3">
         <f>C3/3</f>
-        <v>3000000</v>
+        <v>1233333.3333333333</v>
       </c>
       <c r="E3" s="4">
-        <v>0.245</v>
+        <v>0.25</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C4" s="3">
-        <v>11000000</v>
+        <v>4000000</v>
       </c>
       <c r="D4" s="3">
         <f>C4/3</f>
-        <v>3666666.6666666665</v>
+        <v>1333333.3333333333</v>
       </c>
       <c r="E4" s="4">
-        <v>0.29899999999999999</v>
+        <v>0.27</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C5" s="3">
-        <v>9300000</v>
+        <v>3700000</v>
       </c>
       <c r="D5" s="3">
         <f>C5/3</f>
-        <v>3100000</v>
+        <v>1233333.3333333333</v>
       </c>
       <c r="E5" s="4">
-        <v>0.252</v>
+        <v>0.25</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C6" s="3">
         <f>SUM(C2:C5)</f>
-        <v>36800000</v>
+        <v>14800000</v>
       </c>
       <c r="D6" s="3">
         <f>C6/12</f>
-        <v>3066666.6666666665</v>
+        <v>1233333.3333333333</v>
       </c>
       <c r="E6" s="4">
         <f>SUM(E2:E5)</f>
         <v>1</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1115,117 +1110,117 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{511BA61F-2633-48F8-9DA4-140050B4DB9D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC1ABFCA-0F5A-4D24-9EFD-F9495C6C7E4E}">
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.95" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="33.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16.25" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>